<commit_message>
Receipt cases and other improvements
</commit_message>
<xml_diff>
--- a/excel_test_cases_updated/test_create_invoice_copy.xlsx
+++ b/excel_test_cases_updated/test_create_invoice_copy.xlsx
@@ -1,408 +1,179 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Samit paudel\Downloads\ariba_automation\sap_test_automation\excel_test_cases_updated\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" tabRatio="878" firstSheet="1" activeTab="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" tabRatio="878" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenario Cover Sheet" sheetId="1" r:id="rId1"/>
-    <sheet name="Steps" sheetId="2" r:id="rId2"/>
-    <sheet name="References" sheetId="3" r:id="rId3"/>
+    <sheet name="Scenario Cover Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Steps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="References" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Scenario Metrics " sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Steps!$A$1:$Q$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Steps'!$A$1:$Q$5</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
-  <si>
-    <t xml:space="preserve">Scenario Owner: </t>
-  </si>
-  <si>
-    <t>Test Cycle:</t>
-  </si>
-  <si>
-    <t>Scenario ID:</t>
-  </si>
-  <si>
-    <t>BI_001</t>
-  </si>
-  <si>
-    <t>Test Objective:</t>
-  </si>
-  <si>
-    <t>Create Guided Buying PR and PO in Ariba Buying for enabled supplier.</t>
-  </si>
-  <si>
-    <t>Scenario Description:</t>
-  </si>
-  <si>
-    <t>Long Description Scenario Summary for items to be tested</t>
-  </si>
-  <si>
-    <t>Search catalog for items
-Add items to cart
-Complete requisition details and submit
-Review PR approval flow 
-Confirm PO generation
-Create associated receipt</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Data Requirements</t>
-  </si>
-  <si>
-    <t>Legacy Reference</t>
-  </si>
-  <si>
-    <t>SAP Reference</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prerequisite </t>
-  </si>
-  <si>
-    <t>Key RICEF Objects</t>
-  </si>
-  <si>
-    <t>Master Data Validation</t>
-  </si>
-  <si>
-    <t>SAP PO Post and Validation</t>
-  </si>
-  <si>
-    <t>SAP Invoice to SAP</t>
-  </si>
-  <si>
-    <t>Payment Remitance Validation to Ariba</t>
-  </si>
-  <si>
-    <t>TEST SRIPT &amp; EXECUTION APPROVAL</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Signature</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Scenario Number</t>
-  </si>
-  <si>
-    <t>Step</t>
-  </si>
-  <si>
-    <t>Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description </t>
-  </si>
-  <si>
-    <t>Tcode</t>
-  </si>
-  <si>
-    <t>Test Data / Test Execution</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Step Completed
-Sucessfully</t>
-  </si>
-  <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>FI Impact</t>
-  </si>
-  <si>
-    <t>RICEF Tested</t>
-  </si>
-  <si>
-    <t>TPR #</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Tester/User ID</t>
-  </si>
-  <si>
-    <t>Y or N</t>
-  </si>
-  <si>
-    <t>Scenario No.</t>
-  </si>
-  <si>
-    <t>Section</t>
-  </si>
-  <si>
-    <t>BL_001</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Buyer</t>
-  </si>
-  <si>
-    <t>Logon to Ariba Spend Management to access Ariba Buying using the provided URL.</t>
-  </si>
-  <si>
-    <t>Login
-Password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Garden LEGACY Buying page is presented. </t>
-  </si>
-  <si>
-    <t>Confirm logon to the child realm - Central Garden and Pet Company - C1-TEST is displayed in the upper right corner.  If not, click the globe icon and when displayed, click on the link "Central Garden and Pet Company - C1-TEST"</t>
-  </si>
-  <si>
-    <t>Displayed realm says: "Central Garden and Pet Company - C1-TEST"</t>
-  </si>
-  <si>
-    <t>On Ariba B&amp;I homepage, click on Create &gt; Invoice</t>
-  </si>
-  <si>
-    <t>Invoice creation page is displayed.</t>
-  </si>
-  <si>
-    <t>Invoice Creation</t>
-  </si>
-  <si>
-    <t>AP</t>
-  </si>
-  <si>
-    <t>Enter or  verify the information in the Invoice Entry Header Information.                                                                                                          Note: Only red items should be editable.</t>
-  </si>
-  <si>
-    <t>Type: 
-Supplier: LAKESHORE LEARNING MATERIALS
-Supplier Invoice #: 1234
-Invoice Date: 22/04/2025
-Payment Terms: select
-Ship From: LAKESHORE LEARNING MATERIALS
-Ship To: Ariba - Pittsburgh
-Remit To Address: 1000005900</t>
-  </si>
-  <si>
-    <t>You are able to fill all the necessary details without any error.</t>
-  </si>
-  <si>
-    <t>On line items you can view the details of your line items.
-In Price, enter more than PO price. and click on Update.</t>
-  </si>
-  <si>
-    <t>No: 1, Description: Book Bins - Set of 16, Order_ID: PO192, Qty: 5, Unit: each, Price: $94.50 USD, Amount: $472.50 USD, Discount: , Gross_Amount: $472.50 USD</t>
-  </si>
-  <si>
-    <t>Quantity is set as the same specified in the PO.</t>
-  </si>
-  <si>
-    <t>Click "Submit" at either the top or bottom of the page. Note down the invoice number for future reference.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You are able to submit the invoice without any error.                                                                    Display message: Your request has been submitted for approval. </t>
-  </si>
-  <si>
-    <t>A.Click on View the Status of your request.
-B.Click on reference tab and review all the related documents.</t>
-  </si>
-  <si>
-    <t>Invoice is approved and status at top right is Reconciled.</t>
-  </si>
-  <si>
-    <t>INV76767-732</t>
-  </si>
-  <si>
-    <t>Count of Status</t>
-  </si>
-  <si>
-    <t>(blank)</t>
-  </si>
-  <si>
-    <t>10 - Not Started</t>
-  </si>
-  <si>
-    <t>20 - In-Process</t>
-  </si>
-  <si>
-    <t>30 - TPR Hold</t>
-  </si>
-  <si>
-    <t>40 - DEV Hold</t>
-  </si>
-  <si>
-    <t>50 - Pass</t>
-  </si>
-  <si>
-    <t>60 - N/A</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>PP_018</t>
-  </si>
-  <si>
-    <t>RTR</t>
-  </si>
-  <si>
-    <t>PTP</t>
-  </si>
-  <si>
-    <t>PP</t>
-  </si>
-  <si>
-    <t>IMWM</t>
-  </si>
-  <si>
-    <t>PP_018 Total</t>
-  </si>
-  <si>
-    <t>ZZZ999</t>
-  </si>
-  <si>
-    <t>ZZZ999 Total</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="26">
     <font>
+      <name val="Arial"/>
       <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="8"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="14"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="14"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="10"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF00B0F0"/>
       <sz val="14"/>
-      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <color rgb="FF00B0F0"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FFFF0000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0070C0"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="8">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -444,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="50">
+  <borders count="56">
     <border>
       <left/>
       <right/>
@@ -975,6 +746,19 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -1028,6 +812,55 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -1040,288 +873,353 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="148">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" pivotButton="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" pivotButton="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="1" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" applyAlignment="1" pivotButton="1" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="47" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1524,17 +1422,17 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
@@ -1542,27 +1440,27 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
@@ -1619,25 +1517,18 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Browning G Hollomon" refreshedDate="39386.436179745368" createdVersion="1" refreshedVersion="3" recordCount="137" upgradeOnRefresh="1">
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshedBy="Browning G Hollomon" refreshedDate="39386.43617974537" createdVersion="1" refreshedVersion="3" recordCount="137" upgradeOnRefresh="1" r:id="rId1">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:N13" sheet="SM-MD Tank Final"/>
   </cacheSource>
   <cacheFields count="15">
-    <cacheField name="Scenario Number" numFmtId="0">
-      <sharedItems containsBlank="1" count="28">
+    <cacheField name="Scenario Number" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="28" containsBlank="1">
         <m/>
         <s v="Demand Planning"/>
         <s v="FTS001"/>
@@ -1668,11 +1559,11 @@
         <s v="OTC001" u="1"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Step" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="46"/>
+    <cacheField name="Step" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1" containsInteger="1" containsNumber="1" containsString="0" minValue="1" maxValue="46"/>
     </cacheField>
-    <cacheField name="Team" numFmtId="0">
-      <sharedItems containsBlank="1" count="7">
+    <cacheField name="Team" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="7" containsBlank="1">
         <m/>
         <s v="FTS"/>
         <s v="PTP"/>
@@ -1682,35 +1573,35 @@
         <s v="XXX" u="1"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Description " numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Description " uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Tcode" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Tcode" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Tester" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Tester" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Test Data / Test Execution" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Test Data / Test Execution" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Expected Result" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Expected Result" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Actual Result" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="Actual Result" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="FI Impact" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="FI Impact" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="RICEF Tested" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+    <cacheField name="RICEF Tested" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="TPR #" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    <cacheField name="TPR #" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1" containsNonDate="0" containsString="0"/>
     </cacheField>
-    <cacheField name="Status" numFmtId="0">
-      <sharedItems containsBlank="1" count="34">
+    <cacheField name="Status" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="34" containsBlank="1">
         <m/>
         <s v="50 - Pass"/>
         <s v="60 - N/A"/>
@@ -1747,18 +1638,13 @@
         <s v="20 In Process" u="1"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="User ID" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    <cacheField name="User ID" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1" containsNonDate="0" containsString="0"/>
     </cacheField>
-    <cacheField name="Comments" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    <cacheField name="Comments" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1" containsNonDate="0" containsString="0"/>
     </cacheField>
   </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
 </pivotCacheDefinition>
 </file>
 
@@ -4097,231 +3983,231 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" dataOnRows="1" dataCaption="Data" showError="0" showMissing="1" updatedVersion="3" minRefreshableVersion="0" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="0" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="1" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="0" outline="0" outlineData="0" compactData="0" published="0" gridDropZones="1" immersive="1" multipleFieldFilters="0" chartFormat="0" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
   <location ref="A3:J12" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
   <pivotFields count="15">
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
+    <pivotField axis="axisRow" showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
       <items count="29">
-        <item h="1" m="1" x="27"/>
-        <item h="1" x="0"/>
-        <item h="1" m="1" x="10"/>
-        <item n="PP_018" x="2"/>
-        <item m="1" x="8"/>
-        <item x="7"/>
-        <item m="1" x="16"/>
-        <item m="1" x="18"/>
-        <item m="1" x="20"/>
-        <item m="1" x="22"/>
-        <item m="1" x="23"/>
-        <item m="1" x="24"/>
-        <item m="1" x="25"/>
-        <item m="1" x="26"/>
-        <item m="1" x="9"/>
-        <item m="1" x="11"/>
-        <item m="1" x="12"/>
-        <item m="1" x="13"/>
-        <item m="1" x="14"/>
-        <item m="1" x="15"/>
-        <item m="1" x="17"/>
-        <item m="1" x="19"/>
-        <item m="1" x="21"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item t="default"/>
+        <item t="data" h="1" sd="1" m="1" x="27"/>
+        <item t="data" h="1" sd="1" x="0"/>
+        <item t="data" h="1" sd="1" m="1" x="10"/>
+        <item n="PP_018" t="data" sd="1" x="2"/>
+        <item t="data" sd="1" m="1" x="8"/>
+        <item t="data" sd="1" x="7"/>
+        <item t="data" sd="1" m="1" x="16"/>
+        <item t="data" sd="1" m="1" x="18"/>
+        <item t="data" sd="1" m="1" x="20"/>
+        <item t="data" sd="1" m="1" x="22"/>
+        <item t="data" sd="1" m="1" x="23"/>
+        <item t="data" sd="1" m="1" x="24"/>
+        <item t="data" sd="1" m="1" x="25"/>
+        <item t="data" sd="1" m="1" x="26"/>
+        <item t="data" sd="1" m="1" x="9"/>
+        <item t="data" sd="1" m="1" x="11"/>
+        <item t="data" sd="1" m="1" x="12"/>
+        <item t="data" sd="1" m="1" x="13"/>
+        <item t="data" sd="1" m="1" x="14"/>
+        <item t="data" sd="1" m="1" x="15"/>
+        <item t="data" sd="1" m="1" x="17"/>
+        <item t="data" sd="1" m="1" x="19"/>
+        <item t="data" sd="1" m="1" x="21"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="data" sd="1" x="3"/>
+        <item t="data" sd="1" x="4"/>
+        <item t="data" sd="1" x="5"/>
+        <item t="data" sd="1" x="6"/>
+        <item t="default" sd="1"/>
       </items>
     </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField axis="axisRow" showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
       <items count="8">
-        <item h="1" x="0"/>
-        <item m="1" x="5"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item n="PP" x="1"/>
-        <item m="1" x="6"/>
-        <item x="3"/>
-        <item t="default"/>
+        <item t="data" h="1" sd="1" x="0"/>
+        <item t="data" sd="1" m="1" x="5"/>
+        <item t="data" sd="1" x="4"/>
+        <item t="data" sd="1" x="2"/>
+        <item n="PP" t="data" sd="1" x="1"/>
+        <item t="data" sd="1" m="1" x="6"/>
+        <item t="data" sd="1" x="3"/>
+        <item t="default" sd="1"/>
       </items>
     </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisCol" dataField="1" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField axis="axisCol" dataField="1" showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
       <items count="35">
-        <item m="1" x="12"/>
-        <item m="1" x="16"/>
-        <item m="1" x="29"/>
-        <item m="1" x="31"/>
-        <item m="1" x="24"/>
-        <item x="0"/>
-        <item m="1" x="17"/>
-        <item m="1" x="33"/>
-        <item m="1" x="26"/>
-        <item m="1" x="13"/>
-        <item m="1" x="9"/>
-        <item m="1" x="25"/>
-        <item m="1" x="8"/>
-        <item m="1" x="28"/>
-        <item m="1" x="19"/>
-        <item m="1" x="30"/>
-        <item m="1" x="15"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="10"/>
-        <item m="1" x="18"/>
-        <item m="1" x="11"/>
-        <item m="1" x="22"/>
-        <item m="1" x="32"/>
-        <item m="1" x="20"/>
-        <item m="1" x="27"/>
-        <item m="1" x="14"/>
-        <item m="1" x="23"/>
-        <item m="1" x="7"/>
-        <item m="1" x="21"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
+        <item t="data" sd="1" m="1" x="12"/>
+        <item t="data" sd="1" m="1" x="16"/>
+        <item t="data" sd="1" m="1" x="29"/>
+        <item t="data" sd="1" m="1" x="31"/>
+        <item t="data" sd="1" m="1" x="24"/>
+        <item t="data" sd="1" x="0"/>
+        <item t="data" sd="1" m="1" x="17"/>
+        <item t="data" sd="1" m="1" x="33"/>
+        <item t="data" sd="1" m="1" x="26"/>
+        <item t="data" sd="1" m="1" x="13"/>
+        <item t="data" sd="1" m="1" x="9"/>
+        <item t="data" sd="1" m="1" x="25"/>
+        <item t="data" sd="1" m="1" x="8"/>
+        <item t="data" sd="1" m="1" x="28"/>
+        <item t="data" sd="1" m="1" x="19"/>
+        <item t="data" sd="1" m="1" x="30"/>
+        <item t="data" sd="1" m="1" x="15"/>
+        <item t="data" sd="1" x="3"/>
+        <item t="data" sd="1" x="4"/>
+        <item t="data" sd="1" x="5"/>
+        <item t="data" sd="1" x="6"/>
+        <item t="data" sd="1" m="1" x="10"/>
+        <item t="data" sd="1" m="1" x="18"/>
+        <item t="data" sd="1" m="1" x="11"/>
+        <item t="data" sd="1" m="1" x="22"/>
+        <item t="data" sd="1" m="1" x="32"/>
+        <item t="data" sd="1" m="1" x="20"/>
+        <item t="data" sd="1" m="1" x="27"/>
+        <item t="data" sd="1" m="1" x="14"/>
+        <item t="data" sd="1" m="1" x="23"/>
+        <item t="data" sd="1" m="1" x="7"/>
+        <item t="data" sd="1" m="1" x="21"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="data" sd="1" x="2"/>
+        <item t="default" sd="1"/>
       </items>
     </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="0" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" includeNewItemsInFilter="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
   </pivotFields>
   <rowFields count="2">
     <field x="0"/>
     <field x="2"/>
   </rowFields>
   <rowItems count="8">
-    <i>
+    <i t="data" r="0" i="0">
       <x v="3"/>
       <x v="2"/>
     </i>
-    <i r="1">
+    <i t="data" r="1" i="0">
       <x v="3"/>
     </i>
-    <i r="1">
+    <i t="data" r="1" i="0">
       <x v="4"/>
     </i>
-    <i r="1">
+    <i t="data" r="1" i="0">
       <x v="6"/>
     </i>
-    <i t="default">
+    <i t="default" r="0" i="0">
       <x v="3"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="5"/>
       <x v="4"/>
     </i>
-    <i t="default">
+    <i t="default" r="0" i="0">
       <x v="5"/>
     </i>
-    <i t="grand">
-      <x/>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
     </i>
   </rowItems>
   <colFields count="1">
     <field x="12"/>
   </colFields>
   <colItems count="8">
-    <i>
+    <i t="data" r="0" i="0">
       <x v="5"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="17"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="18"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="19"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="20"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="32"/>
     </i>
-    <i>
+    <i t="data" r="0" i="0">
       <x v="33"/>
     </i>
-    <i t="grand">
-      <x/>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of Status" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of Status" fld="12" subtotal="count" showDataAs="normal" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="44">
-    <format dxfId="43">
-      <pivotArea outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="43">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format action="formatting" dxfId="42">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format action="formatting" dxfId="41">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="40">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="40">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="2" count="0"/>
+          <reference field="2"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="39">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format action="formatting" dxfId="38">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="37">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
-      <pivotArea outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="36">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format action="formatting" dxfId="35">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format action="formatting" dxfId="34">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="33">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="33">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="2" count="0"/>
+          <reference field="2"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="32">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="31">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="30">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format action="formatting" dxfId="29">
       <pivotArea field="12" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format action="formatting" dxfId="28">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="27">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="12" count="5">
+          <reference field="12">
             <x v="6"/>
             <x v="7"/>
             <x v="8"/>
@@ -4331,10 +4217,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
-      <pivotArea outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="26">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="12" count="5" selected="0">
+          <reference field="12" selected="0">
             <x v="6"/>
             <x v="7"/>
             <x v="8"/>
@@ -4344,16 +4230,16 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format action="formatting" dxfId="25">
       <pivotArea field="12" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format action="formatting" dxfId="24">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="23">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="12" count="5">
+          <reference field="12">
             <x v="6"/>
             <x v="7"/>
             <x v="8"/>
@@ -4363,171 +4249,171 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="22">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1">
+          <reference field="0">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="21">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" defaultSubtotal="1">
+          <reference field="0" defaultSubtotal="1">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="20">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
-          <reference field="0" count="1" selected="0">
+          <reference field="0" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="2" count="0"/>
+          <reference field="2"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="19">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1">
+          <reference field="0">
             <x v="2"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="18">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" defaultSubtotal="1">
+          <reference field="0" defaultSubtotal="1">
             <x v="2"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="17">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
-          <reference field="0" count="1" selected="0">
+          <reference field="0" selected="0">
             <x v="2"/>
           </reference>
-          <reference field="2" count="1">
+          <reference field="2">
             <x v="1"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format action="formatting" dxfId="16">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
-      <pivotArea outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="15">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" selected="0" defaultSubtotal="1">
+          <reference field="0" selected="0" defaultSubtotal="1">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="14">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" defaultSubtotal="1">
+          <reference field="0" defaultSubtotal="1">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
-      <pivotArea outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="13">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" selected="0" defaultSubtotal="1">
+          <reference field="0" selected="0" defaultSubtotal="1">
             <x v="3"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
-      <pivotArea outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="12">
+      <pivotArea type="normal" dataOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" selected="0">
+          <reference field="0" selected="0">
             <x v="5"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format action="formatting" dxfId="11">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format action="formatting" dxfId="10">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format action="formatting" dxfId="9">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="8">
+    <format action="formatting" dxfId="8">
       <pivotArea field="12" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format action="formatting" dxfId="7">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="6">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="0"/>
+          <reference field="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="5">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="1" defaultSubtotal="1">
+          <reference field="0" defaultSubtotal="1">
             <x v="3"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="4">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
-          <reference field="0" count="1" selected="0">
+          <reference field="0" selected="0">
             <x v="3"/>
           </reference>
-          <reference field="2" count="0"/>
+          <reference field="2"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="3">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
-          <reference field="0" count="1" selected="0">
+          <reference field="0" selected="0">
             <x v="5"/>
           </reference>
-          <reference field="2" count="2">
+          <reference field="2">
             <x v="4"/>
             <x v="6"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    <format action="formatting" dxfId="2">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="1">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="12" count="0"/>
+          <reference field="12"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+    <format action="formatting" dxfId="0">
+      <pivotArea type="normal" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="12" count="0"/>
+          <reference field="12"/>
         </references>
       </pivotArea>
     </format>
@@ -4822,511 +4708,524 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F70"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="11.4"/>
   <cols>
-    <col min="1" max="2" width="25.88671875" style="38" customWidth="1"/>
-    <col min="3" max="3" width="25" style="38" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" style="38" customWidth="1"/>
-    <col min="5" max="5" width="34.88671875" style="38" customWidth="1"/>
-    <col min="6" max="14" width="40.88671875" style="38" customWidth="1"/>
-    <col min="15" max="15" width="9.109375" style="38" customWidth="1"/>
-    <col min="16" max="16384" width="9.109375" style="38"/>
+    <col width="25.88671875" customWidth="1" style="38" min="1" max="2"/>
+    <col width="25" customWidth="1" style="38" min="3" max="3"/>
+    <col width="25.88671875" customWidth="1" style="38" min="4" max="4"/>
+    <col width="34.88671875" customWidth="1" style="38" min="5" max="5"/>
+    <col width="40.88671875" customWidth="1" style="38" min="6" max="14"/>
+    <col width="9.109375" customWidth="1" style="38" min="15" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="37"/>
-    </row>
-    <row r="2" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="108"/>
-      <c r="C2" s="109"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="40"/>
-    </row>
-    <row r="3" spans="1:6" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="110" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="112"/>
-    </row>
-    <row r="4" spans="1:6" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="110" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="111"/>
-      <c r="D4" s="111"/>
-      <c r="E4" s="112"/>
-    </row>
-    <row r="5" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="113" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="118"/>
-      <c r="C5" s="100"/>
-      <c r="D5" s="100"/>
-      <c r="E5" s="106"/>
-    </row>
-    <row r="6" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="114"/>
-      <c r="B6" s="119"/>
-      <c r="C6" s="119"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="120"/>
-    </row>
-    <row r="7" spans="1:6" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="41"/>
-      <c r="E7" s="42"/>
-    </row>
-    <row r="8" spans="1:6" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="113" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="116"/>
-      <c r="C8" s="116"/>
-      <c r="D8" s="116"/>
-      <c r="E8" s="117"/>
-    </row>
-    <row r="9" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="102" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="103"/>
-      <c r="C9" s="103"/>
-      <c r="D9" s="103"/>
-      <c r="E9" s="104"/>
-    </row>
-    <row r="10" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="105"/>
-      <c r="B10" s="100"/>
-      <c r="C10" s="100"/>
-      <c r="D10" s="100"/>
-      <c r="E10" s="106"/>
-    </row>
-    <row r="11" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="105"/>
-      <c r="B11" s="100"/>
-      <c r="C11" s="100"/>
-      <c r="D11" s="100"/>
-      <c r="E11" s="106"/>
-    </row>
-    <row r="12" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="105"/>
-      <c r="B12" s="100"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="100"/>
-      <c r="E12" s="106"/>
-      <c r="F12" s="38" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="105"/>
-      <c r="B13" s="100"/>
-      <c r="C13" s="100"/>
-      <c r="D13" s="100"/>
-      <c r="E13" s="106"/>
-    </row>
-    <row r="14" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="105"/>
-      <c r="B14" s="100"/>
-      <c r="C14" s="100"/>
-      <c r="D14" s="100"/>
-      <c r="E14" s="106"/>
-    </row>
-    <row r="15" spans="1:6" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="105"/>
-      <c r="B15" s="100"/>
-      <c r="C15" s="100"/>
-      <c r="D15" s="100"/>
-      <c r="E15" s="106"/>
-    </row>
-    <row r="16" spans="1:6" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="44" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="44" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="45"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="63"/>
-      <c r="B17" s="96"/>
-      <c r="C17" s="91"/>
-      <c r="D17" s="107"/>
-      <c r="E17" s="104"/>
-    </row>
-    <row r="18" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="61"/>
-      <c r="B18" s="91"/>
-      <c r="C18" s="91"/>
-      <c r="D18" s="105"/>
-      <c r="E18" s="106"/>
-    </row>
-    <row r="19" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="62"/>
-      <c r="B19" s="91"/>
-      <c r="C19" s="91"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B20" s="91"/>
-      <c r="C20" s="91"/>
-      <c r="D20" s="105"/>
-      <c r="E20" s="106"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B21" s="46"/>
-      <c r="C21" s="91"/>
-      <c r="D21" s="105"/>
-      <c r="E21" s="106"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="95"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="91"/>
-      <c r="D22" s="105"/>
-      <c r="E22" s="106"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="95"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="91"/>
-      <c r="D23" s="105"/>
-      <c r="E23" s="106"/>
-    </row>
-    <row r="24" spans="1:5" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
-      <c r="D24" s="105"/>
-      <c r="E24" s="106"/>
-    </row>
-    <row r="25" spans="1:5" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="45"/>
-    </row>
-    <row r="26" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="99"/>
-      <c r="B26" s="100"/>
-      <c r="C26" s="100"/>
-      <c r="D26" s="100"/>
-      <c r="E26" s="42"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="99"/>
-      <c r="B27" s="100"/>
-      <c r="C27" s="100"/>
-      <c r="D27" s="100"/>
-      <c r="E27" s="42"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="99"/>
-      <c r="B28" s="100"/>
-      <c r="C28" s="100"/>
-      <c r="D28" s="100"/>
-      <c r="E28" s="42"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="99"/>
-      <c r="B29" s="100"/>
-      <c r="C29" s="100"/>
-      <c r="D29" s="100"/>
-      <c r="E29" s="42"/>
-    </row>
-    <row r="30" spans="1:5" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
-      <c r="E30" s="42"/>
-    </row>
-    <row r="31" spans="1:5" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="43" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="45"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="99" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" s="100"/>
-      <c r="C32" s="100"/>
-      <c r="D32" s="100"/>
-      <c r="E32" s="42"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="99" t="s">
-        <v>17</v>
-      </c>
-      <c r="B33" s="100"/>
-      <c r="C33" s="100"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="42"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="99" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="100"/>
-      <c r="C34" s="100"/>
-      <c r="D34" s="100"/>
-      <c r="E34" s="42"/>
-    </row>
-    <row r="35" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="99" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" s="100"/>
-      <c r="C35" s="100"/>
-      <c r="D35" s="100"/>
-      <c r="E35" s="48"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="101"/>
-      <c r="B36" s="100"/>
-      <c r="C36" s="115"/>
-      <c r="D36" s="100"/>
-      <c r="E36" s="42"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="101"/>
-      <c r="B37" s="100"/>
-      <c r="C37" s="115"/>
-      <c r="D37" s="100"/>
-      <c r="E37" s="42"/>
-    </row>
-    <row r="38" spans="1:5" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" s="42"/>
-    </row>
-    <row r="39" spans="1:5" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B39" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="C39" s="51" t="s">
-        <v>23</v>
-      </c>
-      <c r="D39" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" s="45"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="93"/>
-      <c r="B40" s="94"/>
-      <c r="C40" s="94"/>
-      <c r="D40" s="94"/>
-      <c r="E40" s="52"/>
-    </row>
-    <row r="41" spans="1:5" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="53"/>
-      <c r="B41" s="54"/>
-      <c r="C41" s="54"/>
-      <c r="D41" s="54"/>
-      <c r="E41" s="55"/>
-    </row>
-    <row r="43" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="56"/>
-      <c r="B47" s="57"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-    </row>
-    <row r="48" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="56"/>
-      <c r="B48" s="57"/>
-      <c r="C48" s="57"/>
-      <c r="D48" s="57"/>
-    </row>
-    <row r="49" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="58"/>
-      <c r="B49" s="59"/>
-      <c r="C49" s="60"/>
-      <c r="D49" s="59"/>
-      <c r="E49" s="59"/>
-    </row>
-    <row r="50" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="57"/>
-      <c r="B50" s="57"/>
-      <c r="C50" s="57"/>
-      <c r="D50" s="57"/>
-    </row>
-    <row r="51" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="57"/>
-      <c r="B51" s="57"/>
-      <c r="C51" s="57"/>
-      <c r="D51" s="57"/>
-    </row>
-    <row r="52" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="57"/>
-      <c r="B52" s="57"/>
-      <c r="C52" s="57"/>
-      <c r="D52" s="57"/>
-    </row>
-    <row r="53" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="57"/>
-      <c r="B53" s="57"/>
-      <c r="C53" s="57"/>
-      <c r="D53" s="57"/>
-    </row>
-    <row r="54" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="57"/>
-      <c r="B54" s="57"/>
-      <c r="C54" s="57"/>
-      <c r="D54" s="57"/>
-    </row>
-    <row r="55" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="56"/>
-      <c r="B55" s="57"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-    </row>
-    <row r="56" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="56"/>
-      <c r="B56" s="57"/>
-      <c r="C56" s="57"/>
-      <c r="D56" s="57"/>
-    </row>
-    <row r="57" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="57"/>
-      <c r="B57" s="57"/>
-      <c r="C57" s="57"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="57"/>
-    </row>
-    <row r="58" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="57"/>
-      <c r="B58" s="57"/>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="57"/>
-    </row>
-    <row r="59" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="57"/>
-      <c r="B59" s="57"/>
-      <c r="C59" s="57"/>
-      <c r="D59" s="57"/>
-      <c r="E59" s="57"/>
-    </row>
-    <row r="60" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="57"/>
-      <c r="B60" s="57"/>
-      <c r="C60" s="57"/>
-      <c r="D60" s="57"/>
-      <c r="E60" s="57"/>
-    </row>
-    <row r="61" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="57"/>
-      <c r="B61" s="57"/>
-      <c r="C61" s="57"/>
-      <c r="D61" s="57"/>
-      <c r="E61" s="57"/>
-    </row>
-    <row r="62" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="57"/>
-      <c r="B62" s="57"/>
-      <c r="C62" s="57"/>
-      <c r="D62" s="57"/>
-      <c r="E62" s="57"/>
-    </row>
-    <row r="63" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="57"/>
-      <c r="B63" s="57"/>
-      <c r="C63" s="57"/>
-      <c r="D63" s="57"/>
-      <c r="E63" s="57"/>
-    </row>
-    <row r="64" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="57"/>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-    </row>
-    <row r="65" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="57"/>
-      <c r="B65" s="57"/>
-      <c r="C65" s="57"/>
-      <c r="D65" s="57"/>
-      <c r="E65" s="57"/>
-    </row>
-    <row r="66" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="57"/>
-      <c r="B66" s="57"/>
-      <c r="C66" s="57"/>
-      <c r="D66" s="57"/>
-      <c r="E66" s="57"/>
-    </row>
-    <row r="67" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="57"/>
-      <c r="B67" s="57"/>
-      <c r="C67" s="57"/>
-      <c r="D67" s="57"/>
-      <c r="E67" s="57"/>
-    </row>
-    <row r="68" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="57"/>
-      <c r="B68" s="57"/>
-      <c r="C68" s="57"/>
-      <c r="D68" s="57"/>
-      <c r="E68" s="57"/>
-    </row>
-    <row r="69" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="57"/>
-      <c r="B69" s="57"/>
-      <c r="C69" s="57"/>
-      <c r="D69" s="57"/>
-      <c r="E69" s="57"/>
-    </row>
-    <row r="70" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="57"/>
-      <c r="B70" s="57"/>
-      <c r="C70" s="57"/>
-      <c r="D70" s="57"/>
-      <c r="E70" s="57"/>
+    <row r="1" ht="14.1" customHeight="1" thickBot="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scenario Owner: </t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="n"/>
+      <c r="C1" s="36" t="n"/>
+      <c r="D1" s="36" t="n"/>
+      <c r="E1" s="37" t="n"/>
+    </row>
+    <row r="2" ht="14.1" customHeight="1" thickBot="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>Test Cycle:</t>
+        </is>
+      </c>
+      <c r="B2" s="102" t="n"/>
+      <c r="C2" s="128" t="n"/>
+      <c r="D2" s="103" t="n"/>
+      <c r="E2" s="41" t="n"/>
+    </row>
+    <row r="3" ht="12" customHeight="1" thickBot="1">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>Scenario ID:</t>
+        </is>
+      </c>
+      <c r="B3" s="129" t="inlineStr">
+        <is>
+          <t>BI_001</t>
+        </is>
+      </c>
+      <c r="C3" s="130" t="n"/>
+      <c r="D3" s="130" t="n"/>
+      <c r="E3" s="131" t="n"/>
+    </row>
+    <row r="4" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>Test Objective:</t>
+        </is>
+      </c>
+      <c r="B4" s="129" t="inlineStr">
+        <is>
+          <t>Create Guided Buying PR and PO in Ariba Buying for enabled supplier.</t>
+        </is>
+      </c>
+      <c r="C4" s="130" t="n"/>
+      <c r="D4" s="130" t="n"/>
+      <c r="E4" s="131" t="n"/>
+    </row>
+    <row r="5" ht="12" customHeight="1">
+      <c r="A5" s="132" t="inlineStr">
+        <is>
+          <t>Scenario Description:</t>
+        </is>
+      </c>
+      <c r="B5" s="111" t="n"/>
+      <c r="E5" s="133" t="n"/>
+    </row>
+    <row r="6" ht="14.1" customHeight="1" thickBot="1">
+      <c r="A6" s="134" t="n"/>
+      <c r="B6" s="135" t="n"/>
+      <c r="C6" s="135" t="n"/>
+      <c r="D6" s="135" t="n"/>
+      <c r="E6" s="136" t="n"/>
+    </row>
+    <row r="7" ht="12" customHeight="1" thickBot="1">
+      <c r="A7" s="42" t="n"/>
+      <c r="E7" s="43" t="n"/>
+    </row>
+    <row r="8" ht="12.75" customHeight="1" thickBot="1">
+      <c r="A8" s="132" t="inlineStr">
+        <is>
+          <t>Long Description Scenario Summary for items to be tested</t>
+        </is>
+      </c>
+      <c r="B8" s="137" t="n"/>
+      <c r="C8" s="137" t="n"/>
+      <c r="D8" s="137" t="n"/>
+      <c r="E8" s="138" t="n"/>
+    </row>
+    <row r="9" ht="12.75" customHeight="1">
+      <c r="A9" s="139" t="inlineStr">
+        <is>
+          <t>Search catalog for items
+Add items to cart
+Complete requisition details and submit
+Review PR approval flow 
+Confirm PO generation
+Create associated receipt</t>
+        </is>
+      </c>
+      <c r="B9" s="140" t="n"/>
+      <c r="C9" s="140" t="n"/>
+      <c r="D9" s="140" t="n"/>
+      <c r="E9" s="141" t="n"/>
+    </row>
+    <row r="10" ht="12.75" customHeight="1">
+      <c r="A10" s="142" t="n"/>
+      <c r="E10" s="133" t="n"/>
+    </row>
+    <row r="11" ht="12.75" customHeight="1">
+      <c r="A11" s="142" t="n"/>
+      <c r="E11" s="133" t="n"/>
+    </row>
+    <row r="12" ht="12.75" customHeight="1">
+      <c r="A12" s="142" t="n"/>
+      <c r="E12" s="133" t="n"/>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="12.75" customHeight="1">
+      <c r="A13" s="142" t="n"/>
+      <c r="E13" s="133" t="n"/>
+    </row>
+    <row r="14" ht="12.75" customHeight="1">
+      <c r="A14" s="142" t="n"/>
+      <c r="E14" s="133" t="n"/>
+    </row>
+    <row r="15" ht="12.75" customHeight="1" thickBot="1">
+      <c r="A15" s="142" t="n"/>
+      <c r="E15" s="133" t="n"/>
+    </row>
+    <row r="16" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>Data Requirements</t>
+        </is>
+      </c>
+      <c r="B16" s="45" t="inlineStr">
+        <is>
+          <t>Legacy Reference</t>
+        </is>
+      </c>
+      <c r="C16" s="45" t="inlineStr">
+        <is>
+          <t>SAP Reference</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="119" t="n"/>
+      <c r="C17" s="101" t="n"/>
+      <c r="D17" s="143" t="n"/>
+      <c r="E17" s="141" t="n"/>
+    </row>
+    <row r="18" ht="12" customHeight="1">
+      <c r="A18" s="67" t="n"/>
+      <c r="B18" s="101" t="n"/>
+      <c r="C18" s="101" t="n"/>
+      <c r="D18" s="142" t="n"/>
+      <c r="E18" s="133" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="68" t="n"/>
+      <c r="B19" s="101" t="n"/>
+      <c r="C19" s="101" t="n"/>
+      <c r="D19" s="142" t="n"/>
+      <c r="E19" s="133" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="101" t="n"/>
+      <c r="C20" s="101" t="n"/>
+      <c r="D20" s="142" t="n"/>
+      <c r="E20" s="133" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="50" t="n"/>
+      <c r="C21" s="101" t="n"/>
+      <c r="D21" s="142" t="n"/>
+      <c r="E21" s="133" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="118" t="n"/>
+      <c r="B22" s="119" t="n"/>
+      <c r="C22" s="101" t="n"/>
+      <c r="D22" s="142" t="n"/>
+      <c r="E22" s="133" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="118" t="n"/>
+      <c r="B23" s="119" t="n"/>
+      <c r="C23" s="101" t="n"/>
+      <c r="D23" s="142" t="n"/>
+      <c r="E23" s="133" t="n"/>
+    </row>
+    <row r="24" ht="12" customHeight="1" thickBot="1">
+      <c r="A24" s="51" t="n"/>
+      <c r="D24" s="142" t="n"/>
+      <c r="E24" s="133" t="n"/>
+    </row>
+    <row r="25" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prerequisite </t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="n"/>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="45" t="n"/>
+      <c r="E25" s="46" t="n"/>
+    </row>
+    <row r="26" ht="12" customHeight="1">
+      <c r="A26" s="100" t="n"/>
+      <c r="E26" s="43" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="100" t="n"/>
+      <c r="E27" s="43" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="100" t="n"/>
+      <c r="E28" s="43" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="100" t="n"/>
+      <c r="E29" s="43" t="n"/>
+    </row>
+    <row r="30" ht="12" customHeight="1" thickBot="1">
+      <c r="A30" s="51" t="n"/>
+      <c r="E30" s="43" t="n"/>
+    </row>
+    <row r="31" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A31" s="44" t="inlineStr">
+        <is>
+          <t>Key RICEF Objects</t>
+        </is>
+      </c>
+      <c r="B31" s="45" t="n"/>
+      <c r="C31" s="45" t="n"/>
+      <c r="D31" s="45" t="n"/>
+      <c r="E31" s="46" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="100" t="inlineStr">
+        <is>
+          <t>Master Data Validation</t>
+        </is>
+      </c>
+      <c r="E32" s="43" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="100" t="inlineStr">
+        <is>
+          <t>SAP PO Post and Validation</t>
+        </is>
+      </c>
+      <c r="E33" s="43" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="100" t="inlineStr">
+        <is>
+          <t>SAP Invoice to SAP</t>
+        </is>
+      </c>
+      <c r="E34" s="43" t="n"/>
+    </row>
+    <row r="35" ht="12.75" customHeight="1">
+      <c r="A35" s="100" t="inlineStr">
+        <is>
+          <t>Payment Remitance Validation to Ariba</t>
+        </is>
+      </c>
+      <c r="E35" s="52" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="98" t="n"/>
+      <c r="C36" s="99" t="n"/>
+      <c r="E36" s="43" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="98" t="n"/>
+      <c r="C37" s="99" t="n"/>
+      <c r="E37" s="43" t="n"/>
+    </row>
+    <row r="38" ht="12" customHeight="1" thickBot="1">
+      <c r="A38" s="53" t="inlineStr">
+        <is>
+          <t>TEST SRIPT &amp; EXECUTION APPROVAL</t>
+        </is>
+      </c>
+      <c r="E38" s="43" t="n"/>
+    </row>
+    <row r="39" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B39" s="55" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C39" s="55" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D39" s="55" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="E39" s="46" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="115" t="n"/>
+      <c r="B40" s="116" t="n"/>
+      <c r="C40" s="116" t="n"/>
+      <c r="D40" s="116" t="n"/>
+      <c r="E40" s="58" t="n"/>
+    </row>
+    <row r="41" ht="12.6" customHeight="1" thickBot="1">
+      <c r="A41" s="59" t="n"/>
+      <c r="B41" s="60" t="n"/>
+      <c r="C41" s="60" t="n"/>
+      <c r="D41" s="60" t="n"/>
+      <c r="E41" s="61" t="n"/>
+    </row>
+    <row r="43" ht="12.75" customHeight="1"/>
+    <row r="44" ht="12.75" customHeight="1"/>
+    <row r="45" ht="12" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="62" t="n"/>
+      <c r="B47" s="63" t="n"/>
+      <c r="C47" s="63" t="n"/>
+      <c r="D47" s="63" t="n"/>
+    </row>
+    <row r="48" ht="12.75" customHeight="1">
+      <c r="A48" s="62" t="n"/>
+      <c r="B48" s="63" t="n"/>
+      <c r="C48" s="63" t="n"/>
+      <c r="D48" s="63" t="n"/>
+    </row>
+    <row r="49" ht="13.2" customHeight="1">
+      <c r="A49" s="64" t="n"/>
+      <c r="B49" s="65" t="n"/>
+      <c r="C49" s="66" t="n"/>
+      <c r="D49" s="65" t="n"/>
+      <c r="E49" s="65" t="n"/>
+    </row>
+    <row r="50" ht="13.2" customHeight="1">
+      <c r="A50" s="63" t="n"/>
+      <c r="B50" s="63" t="n"/>
+      <c r="C50" s="63" t="n"/>
+      <c r="D50" s="63" t="n"/>
+    </row>
+    <row r="51" ht="13.2" customHeight="1">
+      <c r="A51" s="63" t="n"/>
+      <c r="B51" s="63" t="n"/>
+      <c r="C51" s="63" t="n"/>
+      <c r="D51" s="63" t="n"/>
+    </row>
+    <row r="52" ht="13.2" customHeight="1">
+      <c r="A52" s="63" t="n"/>
+      <c r="B52" s="63" t="n"/>
+      <c r="C52" s="63" t="n"/>
+      <c r="D52" s="63" t="n"/>
+    </row>
+    <row r="53" ht="13.2" customHeight="1">
+      <c r="A53" s="63" t="n"/>
+      <c r="B53" s="63" t="n"/>
+      <c r="C53" s="63" t="n"/>
+      <c r="D53" s="63" t="n"/>
+    </row>
+    <row r="54" ht="13.2" customHeight="1">
+      <c r="A54" s="63" t="n"/>
+      <c r="B54" s="63" t="n"/>
+      <c r="C54" s="63" t="n"/>
+      <c r="D54" s="63" t="n"/>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="62" t="n"/>
+      <c r="B55" s="63" t="n"/>
+      <c r="C55" s="63" t="n"/>
+      <c r="D55" s="63" t="n"/>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="62" t="n"/>
+      <c r="B56" s="63" t="n"/>
+      <c r="C56" s="63" t="n"/>
+      <c r="D56" s="63" t="n"/>
+    </row>
+    <row r="57" ht="13.2" customHeight="1">
+      <c r="A57" s="63" t="n"/>
+      <c r="B57" s="63" t="n"/>
+      <c r="C57" s="63" t="n"/>
+      <c r="D57" s="63" t="n"/>
+      <c r="E57" s="63" t="n"/>
+    </row>
+    <row r="58" ht="13.2" customHeight="1">
+      <c r="A58" s="63" t="n"/>
+      <c r="B58" s="63" t="n"/>
+      <c r="C58" s="63" t="n"/>
+      <c r="D58" s="63" t="n"/>
+      <c r="E58" s="63" t="n"/>
+    </row>
+    <row r="59" ht="13.2" customHeight="1">
+      <c r="A59" s="63" t="n"/>
+      <c r="B59" s="63" t="n"/>
+      <c r="C59" s="63" t="n"/>
+      <c r="D59" s="63" t="n"/>
+      <c r="E59" s="63" t="n"/>
+    </row>
+    <row r="60" ht="13.2" customHeight="1">
+      <c r="A60" s="63" t="n"/>
+      <c r="B60" s="63" t="n"/>
+      <c r="C60" s="63" t="n"/>
+      <c r="D60" s="63" t="n"/>
+      <c r="E60" s="63" t="n"/>
+    </row>
+    <row r="61" ht="13.2" customHeight="1">
+      <c r="A61" s="63" t="n"/>
+      <c r="B61" s="63" t="n"/>
+      <c r="C61" s="63" t="n"/>
+      <c r="D61" s="63" t="n"/>
+      <c r="E61" s="63" t="n"/>
+    </row>
+    <row r="62" ht="13.2" customHeight="1">
+      <c r="A62" s="63" t="n"/>
+      <c r="B62" s="63" t="n"/>
+      <c r="C62" s="63" t="n"/>
+      <c r="D62" s="63" t="n"/>
+      <c r="E62" s="63" t="n"/>
+    </row>
+    <row r="63" ht="13.2" customHeight="1">
+      <c r="A63" s="63" t="n"/>
+      <c r="B63" s="63" t="n"/>
+      <c r="C63" s="63" t="n"/>
+      <c r="D63" s="63" t="n"/>
+      <c r="E63" s="63" t="n"/>
+    </row>
+    <row r="64" ht="13.2" customHeight="1">
+      <c r="A64" s="63" t="n"/>
+      <c r="B64" s="63" t="n"/>
+      <c r="C64" s="63" t="n"/>
+      <c r="D64" s="63" t="n"/>
+      <c r="E64" s="63" t="n"/>
+    </row>
+    <row r="65" ht="13.2" customHeight="1">
+      <c r="A65" s="63" t="n"/>
+      <c r="B65" s="63" t="n"/>
+      <c r="C65" s="63" t="n"/>
+      <c r="D65" s="63" t="n"/>
+      <c r="E65" s="63" t="n"/>
+    </row>
+    <row r="66" ht="13.2" customHeight="1">
+      <c r="A66" s="63" t="n"/>
+      <c r="B66" s="63" t="n"/>
+      <c r="C66" s="63" t="n"/>
+      <c r="D66" s="63" t="n"/>
+      <c r="E66" s="63" t="n"/>
+    </row>
+    <row r="67" ht="13.2" customHeight="1">
+      <c r="A67" s="63" t="n"/>
+      <c r="B67" s="63" t="n"/>
+      <c r="C67" s="63" t="n"/>
+      <c r="D67" s="63" t="n"/>
+      <c r="E67" s="63" t="n"/>
+    </row>
+    <row r="68" ht="13.2" customHeight="1">
+      <c r="A68" s="63" t="n"/>
+      <c r="B68" s="63" t="n"/>
+      <c r="C68" s="63" t="n"/>
+      <c r="D68" s="63" t="n"/>
+      <c r="E68" s="63" t="n"/>
+    </row>
+    <row r="69" ht="13.2" customHeight="1">
+      <c r="A69" s="63" t="n"/>
+      <c r="B69" s="63" t="n"/>
+      <c r="C69" s="63" t="n"/>
+      <c r="D69" s="63" t="n"/>
+      <c r="E69" s="63" t="n"/>
+    </row>
+    <row r="70" ht="13.2" customHeight="1">
+      <c r="A70" s="63" t="n"/>
+      <c r="B70" s="63" t="n"/>
+      <c r="C70" s="63" t="n"/>
+      <c r="D70" s="63" t="n"/>
+      <c r="E70" s="63" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A9:E15"/>
+    <mergeCell ref="D17:E24"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="A34:D34"/>
@@ -5341,388 +5240,487 @@
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A9:E15"/>
-    <mergeCell ref="D17:E24"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:E2">
+    <dataValidation sqref="D2:E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"R4-Cycle 1,R4-Cycle 2,R4-Cycle 3,R4-Cycle 4,R4-Regression Test,R4-Business Simulation"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup scale="69" orientation="landscape"/>
+  <pageSetup orientation="landscape" scale="69"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R10"/>
-  <sheetFormatPr defaultColWidth="35.6640625" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="35.6640625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" style="66" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="66" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="64" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" style="64" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" style="66" customWidth="1"/>
-    <col min="6" max="6" width="71.6640625" style="67" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" style="67" customWidth="1"/>
-    <col min="8" max="8" width="56.5546875" style="64" customWidth="1"/>
-    <col min="9" max="9" width="46.44140625" style="64" customWidth="1"/>
-    <col min="10" max="10" width="19.5546875" style="64" customWidth="1"/>
-    <col min="11" max="11" width="25.33203125" style="64" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" style="66" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" style="64" customWidth="1"/>
-    <col min="14" max="14" width="17.44140625" style="64" customWidth="1"/>
-    <col min="15" max="15" width="16.44140625" style="67" customWidth="1"/>
-    <col min="16" max="16" width="13.33203125" style="67" customWidth="1"/>
-    <col min="17" max="17" width="37.109375" style="64" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="35.6640625" style="64" customWidth="1"/>
-    <col min="19" max="16384" width="35.6640625" style="64"/>
+    <col width="10.33203125" customWidth="1" style="72" min="1" max="1"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" style="72" min="2" max="2"/>
+    <col width="10.33203125" customWidth="1" style="70" min="3" max="3"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" style="70" min="4" max="4"/>
+    <col width="14" customWidth="1" style="72" min="5" max="5"/>
+    <col width="71.6640625" customWidth="1" style="73" min="6" max="6"/>
+    <col width="14.109375" customWidth="1" style="73" min="7" max="7"/>
+    <col width="56.5546875" customWidth="1" style="70" min="8" max="8"/>
+    <col width="46.44140625" customWidth="1" style="70" min="9" max="9"/>
+    <col width="19.5546875" customWidth="1" style="70" min="10" max="10"/>
+    <col width="25.33203125" bestFit="1" customWidth="1" style="70" min="11" max="11"/>
+    <col width="18.88671875" customWidth="1" style="72" min="12" max="12"/>
+    <col width="18.6640625" customWidth="1" style="70" min="13" max="13"/>
+    <col width="17.44140625" customWidth="1" style="70" min="14" max="14"/>
+    <col width="16.44140625" customWidth="1" style="73" min="15" max="15"/>
+    <col width="13.33203125" customWidth="1" style="73" min="16" max="16"/>
+    <col width="37.109375" bestFit="1" customWidth="1" style="70" min="17" max="17"/>
+    <col width="35.6640625" customWidth="1" style="70" min="18" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="121" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="121" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" s="97"/>
-      <c r="E1" s="121" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="121" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="121" t="s">
-        <v>29</v>
-      </c>
-      <c r="I1" s="121" t="s">
-        <v>30</v>
-      </c>
-      <c r="J1" s="123" t="s">
-        <v>31</v>
-      </c>
-      <c r="K1" s="121" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" s="97" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" s="121" t="s">
-        <v>34</v>
-      </c>
-      <c r="N1" s="121" t="s">
-        <v>35</v>
-      </c>
-      <c r="O1" s="121" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" s="125" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" s="121" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="122"/>
-      <c r="B2" s="97"/>
-      <c r="C2" s="122"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="124"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="71" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="126"/>
-      <c r="Q2" s="122"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="72"/>
-      <c r="B3" s="72" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="72"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="72"/>
-      <c r="L3" s="72"/>
-      <c r="M3" s="72"/>
-      <c r="N3" s="72"/>
-      <c r="O3" s="75"/>
-      <c r="P3" s="75"/>
-      <c r="Q3" s="72"/>
-    </row>
-    <row r="4" spans="1:18" s="65" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="68" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68">
-        <f t="shared" ref="C4:C10" si="0">ROW(A4)-3</f>
-        <v>1</v>
-      </c>
-      <c r="D4" s="78" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="79" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="78" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="78"/>
-      <c r="H4" s="80" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="78" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" s="77" t="b">
+    <row r="1">
+      <c r="A1" s="124" t="inlineStr">
+        <is>
+          <t>Scenario Number</t>
+        </is>
+      </c>
+      <c r="B1" s="124" t="n"/>
+      <c r="C1" s="124" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D1" s="124" t="n"/>
+      <c r="E1" s="124" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="F1" s="124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description </t>
+        </is>
+      </c>
+      <c r="G1" s="124" t="inlineStr">
+        <is>
+          <t>Tcode</t>
+        </is>
+      </c>
+      <c r="H1" s="124" t="inlineStr">
+        <is>
+          <t>Test Data / Test Execution</t>
+        </is>
+      </c>
+      <c r="I1" s="124" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="J1" s="126" t="inlineStr">
+        <is>
+          <t>Step Completed
+Sucessfully</t>
+        </is>
+      </c>
+      <c r="K1" s="124" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="L1" s="124" t="inlineStr">
+        <is>
+          <t>FI Impact</t>
+        </is>
+      </c>
+      <c r="M1" s="124" t="inlineStr">
+        <is>
+          <t>RICEF Tested</t>
+        </is>
+      </c>
+      <c r="N1" s="124" t="inlineStr">
+        <is>
+          <t>TPR #</t>
+        </is>
+      </c>
+      <c r="O1" s="124" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="P1" s="125" t="inlineStr">
+        <is>
+          <t>Tester/User ID</t>
+        </is>
+      </c>
+      <c r="Q1" s="124" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="51" customHeight="1">
+      <c r="A2" s="144" t="n"/>
+      <c r="B2" s="124" t="n"/>
+      <c r="C2" s="144" t="n"/>
+      <c r="D2" s="78" t="n"/>
+      <c r="E2" s="144" t="n"/>
+      <c r="F2" s="144" t="n"/>
+      <c r="G2" s="144" t="n"/>
+      <c r="H2" s="144" t="n"/>
+      <c r="I2" s="144" t="n"/>
+      <c r="J2" s="145" t="n"/>
+      <c r="K2" s="144" t="n"/>
+      <c r="L2" s="78" t="inlineStr">
+        <is>
+          <t>Y or N</t>
+        </is>
+      </c>
+      <c r="M2" s="144" t="n"/>
+      <c r="N2" s="144" t="n"/>
+      <c r="O2" s="144" t="n"/>
+      <c r="P2" s="146" t="n"/>
+      <c r="Q2" s="144" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="79" t="n"/>
+      <c r="B3" s="79" t="inlineStr">
+        <is>
+          <t>Scenario No.</t>
+        </is>
+      </c>
+      <c r="C3" s="79" t="n"/>
+      <c r="D3" s="79" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="E3" s="79" t="n"/>
+      <c r="F3" s="80" t="n"/>
+      <c r="G3" s="81" t="n"/>
+      <c r="H3" s="81" t="n"/>
+      <c r="I3" s="81" t="n"/>
+      <c r="J3" s="81" t="n"/>
+      <c r="K3" s="79" t="n"/>
+      <c r="L3" s="79" t="n"/>
+      <c r="M3" s="79" t="n"/>
+      <c r="N3" s="79" t="n"/>
+      <c r="O3" s="82" t="n"/>
+      <c r="P3" s="82" t="n"/>
+      <c r="Q3" s="79" t="n"/>
+    </row>
+    <row r="4" ht="36" customFormat="1" customHeight="1" s="71">
+      <c r="A4" s="74" t="inlineStr">
+        <is>
+          <t>BL_001</t>
+        </is>
+      </c>
+      <c r="B4" s="74" t="n"/>
+      <c r="C4" s="74">
+        <f>ROW(A4)-3</f>
+        <v/>
+      </c>
+      <c r="D4" s="85" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E4" s="86" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="F4" s="85" t="inlineStr">
+        <is>
+          <t>Logon to Ariba Spend Management to access Ariba Buying using the provided URL.</t>
+        </is>
+      </c>
+      <c r="G4" s="85" t="n"/>
+      <c r="H4" s="87" t="inlineStr">
+        <is>
+          <t>Login
+Password</t>
+        </is>
+      </c>
+      <c r="I4" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Central Garden LEGACY Buying page is presented. </t>
+        </is>
+      </c>
+      <c r="J4" s="84" t="b">
         <v>0</v>
       </c>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="68"/>
-    </row>
-    <row r="5" spans="1:18" s="65" customFormat="1" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="68"/>
-      <c r="B5" s="68"/>
-      <c r="C5" s="68">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="D5" s="78" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="79" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="78" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="78"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="78" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" s="77" t="b">
+      <c r="K4" s="74" t="n"/>
+      <c r="L4" s="74" t="n"/>
+      <c r="M4" s="74" t="n"/>
+      <c r="N4" s="74" t="n"/>
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="74" t="n"/>
+      <c r="Q4" s="74" t="n"/>
+    </row>
+    <row r="5" ht="195.75" customFormat="1" customHeight="1" s="71">
+      <c r="A5" s="74" t="n"/>
+      <c r="B5" s="74" t="n"/>
+      <c r="C5" s="74">
+        <f>ROW(A5)-3</f>
+        <v/>
+      </c>
+      <c r="D5" s="85" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E5" s="86" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="F5" s="85" t="inlineStr">
+        <is>
+          <t>Confirm logon to the child realm - Central Garden and Pet Company - C1-TEST is displayed in the upper right corner.  If not, click the globe icon and when displayed, click on the link "Central Garden and Pet Company - C1-TEST"</t>
+        </is>
+      </c>
+      <c r="G5" s="85" t="n"/>
+      <c r="H5" s="88" t="n"/>
+      <c r="I5" s="85" t="inlineStr">
+        <is>
+          <t>Displayed realm says: "Central Garden and Pet Company - C1-TEST"</t>
+        </is>
+      </c>
+      <c r="J5" s="84" t="b">
         <v>0</v>
       </c>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="68"/>
-      <c r="O5" s="68"/>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-    </row>
-    <row r="6" spans="1:18" s="65" customFormat="1" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="68"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="D6" s="78" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" s="79" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="98" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="98" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="77"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
-      <c r="N6" s="68"/>
-      <c r="O6" s="68"/>
-      <c r="P6" s="68"/>
-      <c r="Q6" s="68"/>
-    </row>
-    <row r="7" spans="1:18" s="70" customFormat="1" ht="306" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="76"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="76">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="D7" s="83" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="85" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="82"/>
-      <c r="H7" s="84" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="85" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="77" t="b">
+      <c r="K5" s="74" t="n"/>
+      <c r="L5" s="74" t="n"/>
+      <c r="M5" s="74" t="n"/>
+      <c r="N5" s="74" t="n"/>
+      <c r="O5" s="74" t="n"/>
+      <c r="P5" s="74" t="n"/>
+      <c r="Q5" s="74" t="n"/>
+    </row>
+    <row r="6" ht="195.75" customFormat="1" customHeight="1" s="71">
+      <c r="A6" s="74" t="n"/>
+      <c r="B6" s="74" t="n"/>
+      <c r="C6" s="74">
+        <f>ROW(A6)-3</f>
+        <v/>
+      </c>
+      <c r="D6" s="85" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="F6" s="127" t="inlineStr">
+        <is>
+          <t>On Ariba B&amp;I homepage, click on Create &gt; Invoice</t>
+        </is>
+      </c>
+      <c r="G6" s="85" t="n"/>
+      <c r="H6" s="88" t="n"/>
+      <c r="I6" s="127" t="inlineStr">
+        <is>
+          <t>Invoice creation page is displayed.</t>
+        </is>
+      </c>
+      <c r="J6" s="84" t="n"/>
+      <c r="K6" s="74" t="n"/>
+      <c r="L6" s="74" t="n"/>
+      <c r="M6" s="74" t="n"/>
+      <c r="N6" s="74" t="n"/>
+      <c r="O6" s="74" t="n"/>
+      <c r="P6" s="74" t="n"/>
+      <c r="Q6" s="74" t="n"/>
+    </row>
+    <row r="7" ht="306" customFormat="1" customHeight="1" s="76">
+      <c r="A7" s="83" t="n"/>
+      <c r="B7" s="83" t="n"/>
+      <c r="C7" s="83">
+        <f>ROW(A7)-3</f>
+        <v/>
+      </c>
+      <c r="D7" s="90" t="inlineStr">
+        <is>
+          <t>Invoice Creation</t>
+        </is>
+      </c>
+      <c r="E7" s="92" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="F7" s="90" t="inlineStr">
+        <is>
+          <t>Enter or  verify the information in the Invoice Entry Header Information.                                                                                                          Note: Only red items should be editable.</t>
+        </is>
+      </c>
+      <c r="G7" s="89" t="n"/>
+      <c r="H7" s="147" t="inlineStr">
+        <is>
+          <t>Type: 
+Supplier: LAKESHORE LEARNING MATERIALS
+Supplier Invoice #: 1234454545
+Invoice Date: Tue, 22 Apr, 2025
+Payment Terms: select
+Ship From: LAKESHORE LEARNING MATERIALS
+Ship To: Ariba - Pittsburgh
+Remit To Address: 2695 EAST DOMINGUEZ STREET</t>
+        </is>
+      </c>
+      <c r="I7" s="92" t="inlineStr">
+        <is>
+          <t>You are able to fill all the necessary details without any error.</t>
+        </is>
+      </c>
+      <c r="J7" s="84" t="b">
         <v>0</v>
       </c>
-      <c r="K7" s="76"/>
-      <c r="L7" s="76"/>
-      <c r="M7" s="76"/>
-      <c r="N7" s="76"/>
-      <c r="O7" s="76"/>
-      <c r="P7" s="76"/>
-      <c r="Q7" s="76"/>
-      <c r="R7" s="69"/>
-    </row>
-    <row r="8" spans="1:18" s="70" customFormat="1" ht="163.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="76"/>
-      <c r="B8" s="76"/>
-      <c r="C8" s="76">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D8" s="85" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="85" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="84" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" s="85"/>
-      <c r="H8" s="84" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="85" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" s="77" t="b">
+      <c r="K7" s="83" t="n"/>
+      <c r="L7" s="83" t="n"/>
+      <c r="M7" s="83" t="n"/>
+      <c r="N7" s="83" t="n"/>
+      <c r="O7" s="83" t="n"/>
+      <c r="P7" s="83" t="n"/>
+      <c r="Q7" s="83" t="n"/>
+      <c r="R7" s="75" t="n"/>
+    </row>
+    <row r="8" ht="163.5" customFormat="1" customHeight="1" s="76">
+      <c r="A8" s="83" t="n"/>
+      <c r="B8" s="83" t="n"/>
+      <c r="C8" s="83">
+        <f>ROW(A8)-3</f>
+        <v/>
+      </c>
+      <c r="D8" s="92" t="inlineStr">
+        <is>
+          <t>Invoice Creation</t>
+        </is>
+      </c>
+      <c r="E8" s="92" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="F8" s="91" t="inlineStr">
+        <is>
+          <t>On line items you can view the details of your line items.
+In Price, enter more than PO price. and click on Update.</t>
+        </is>
+      </c>
+      <c r="G8" s="92" t="n"/>
+      <c r="H8" s="147" t="inlineStr"/>
+      <c r="I8" s="92" t="inlineStr">
+        <is>
+          <t>Quantity is set as the same specified in the PO.</t>
+        </is>
+      </c>
+      <c r="J8" s="84" t="b">
         <v>0</v>
       </c>
-      <c r="K8" s="76"/>
-      <c r="L8" s="76"/>
-      <c r="M8" s="76"/>
-      <c r="N8" s="76"/>
-      <c r="O8" s="76"/>
-      <c r="P8" s="76"/>
-      <c r="Q8" s="76"/>
-      <c r="R8" s="69"/>
-    </row>
-    <row r="9" spans="1:18" s="70" customFormat="1" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="76"/>
-      <c r="B9" s="76"/>
-      <c r="C9" s="76">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="D9" s="85" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="85" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" s="84" t="s">
-        <v>59</v>
-      </c>
-      <c r="G9" s="85"/>
-      <c r="H9" s="85"/>
-      <c r="I9" s="84" t="s">
-        <v>60</v>
-      </c>
-      <c r="J9" s="77" t="b">
+      <c r="K8" s="83" t="n"/>
+      <c r="L8" s="83" t="n"/>
+      <c r="M8" s="83" t="n"/>
+      <c r="N8" s="83" t="n"/>
+      <c r="O8" s="83" t="n"/>
+      <c r="P8" s="83" t="n"/>
+      <c r="Q8" s="83" t="n"/>
+      <c r="R8" s="75" t="n"/>
+    </row>
+    <row r="9" ht="109.5" customFormat="1" customHeight="1" s="76">
+      <c r="A9" s="83" t="n"/>
+      <c r="B9" s="83" t="n"/>
+      <c r="C9" s="83">
+        <f>ROW(A9)-3</f>
+        <v/>
+      </c>
+      <c r="D9" s="92" t="inlineStr">
+        <is>
+          <t>Invoice Creation</t>
+        </is>
+      </c>
+      <c r="E9" s="92" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="F9" s="91" t="inlineStr">
+        <is>
+          <t>Click "Submit" at either the top or bottom of the page. Note down the invoice number for future reference.</t>
+        </is>
+      </c>
+      <c r="G9" s="92" t="n"/>
+      <c r="H9" s="92" t="n"/>
+      <c r="I9" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are able to submit the invoice without any error.                                                                    Display message: Your request has been submitted for approval. </t>
+        </is>
+      </c>
+      <c r="J9" s="84" t="b">
         <v>0</v>
       </c>
-      <c r="K9" s="76"/>
-      <c r="L9" s="76"/>
-      <c r="M9" s="76"/>
-      <c r="N9" s="76"/>
-      <c r="O9" s="76"/>
-      <c r="P9" s="76"/>
-      <c r="Q9" s="76"/>
-      <c r="R9" s="69"/>
-    </row>
-    <row r="10" spans="1:18" s="70" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="88"/>
-      <c r="B10" s="88"/>
-      <c r="C10" s="88">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="D10" s="86" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="86" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="87" t="s">
-        <v>61</v>
-      </c>
-      <c r="G10" s="86"/>
-      <c r="H10" s="86"/>
-      <c r="I10" s="87" t="s">
-        <v>62</v>
-      </c>
-      <c r="J10" s="89" t="b">
+      <c r="K9" s="83" t="n"/>
+      <c r="L9" s="83" t="n"/>
+      <c r="M9" s="83" t="n"/>
+      <c r="N9" s="83" t="n"/>
+      <c r="O9" s="83" t="n"/>
+      <c r="P9" s="83" t="n"/>
+      <c r="Q9" s="83" t="n"/>
+      <c r="R9" s="75" t="n"/>
+    </row>
+    <row r="10" ht="60" customFormat="1" customHeight="1" s="76">
+      <c r="A10" s="95" t="n"/>
+      <c r="B10" s="95" t="n"/>
+      <c r="C10" s="95">
+        <f>ROW(A10)-3</f>
+        <v/>
+      </c>
+      <c r="D10" s="93" t="inlineStr">
+        <is>
+          <t>Invoice Creation</t>
+        </is>
+      </c>
+      <c r="E10" s="93" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="F10" s="94" t="inlineStr">
+        <is>
+          <t>A.Click on View the Status of your request.
+B.Click on reference tab and review all the related documents.</t>
+        </is>
+      </c>
+      <c r="G10" s="93" t="n"/>
+      <c r="H10" s="93" t="n"/>
+      <c r="I10" s="94" t="inlineStr">
+        <is>
+          <t>Invoice is approved and status at top right is Reconciled.</t>
+        </is>
+      </c>
+      <c r="J10" s="96" t="b">
         <v>0</v>
       </c>
-      <c r="K10" s="88" t="s">
-        <v>63</v>
-      </c>
-      <c r="L10" s="88"/>
-      <c r="M10" s="88"/>
-      <c r="N10" s="88"/>
-      <c r="O10" s="88"/>
-      <c r="P10" s="88"/>
-      <c r="Q10" s="88"/>
-      <c r="R10" s="90"/>
+      <c r="K10" s="95" t="inlineStr">
+        <is>
+          <t>INV76767-732</t>
+        </is>
+      </c>
+      <c r="L10" s="95" t="n"/>
+      <c r="M10" s="95" t="n"/>
+      <c r="N10" s="95" t="n"/>
+      <c r="O10" s="95" t="n"/>
+      <c r="P10" s="95" t="n"/>
+      <c r="Q10" s="95" t="n"/>
+      <c r="R10" s="97" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q5"/>
   <mergeCells count="14">
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="O1:O2"/>
-    <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="N1:N2"/>
@@ -5734,285 +5732,373 @@
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="J1:J2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L10 O4:O6">
+    <dataValidation sqref="L7:L10 O4:O6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"10 - Not Started,20 - In-Process,30 - TPR Hold,40 - DEV Hold,50 - Pass,60 - N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4:L6">
+    <dataValidation sqref="L4:L6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E6">
+    <dataValidation sqref="E4:E6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AP,Buyer,PO Approv,Inv Approv,Watcher,SAP Tech Team,Prem Tech,Prem Funct"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.45" right="0.45" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="61" fitToHeight="10" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" scale="61" fitToHeight="10" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.44140625" defaultRowHeight="13.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:J12"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:R46"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="17.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.44140625" style="2" customWidth="1"/>
-    <col min="3" max="7" width="14.33203125" style="2" customWidth="1"/>
-    <col min="8" max="9" width="14.33203125" style="1" customWidth="1"/>
-    <col min="10" max="11" width="11.6640625" style="1" customWidth="1"/>
-    <col min="12" max="17" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.109375" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.109375" style="1"/>
+    <col width="14.88671875" customWidth="1" style="2" min="1" max="1"/>
+    <col width="8.44140625" customWidth="1" style="2" min="2" max="2"/>
+    <col width="14.33203125" customWidth="1" style="2" min="3" max="7"/>
+    <col width="14.33203125" customWidth="1" style="1" min="8" max="9"/>
+    <col width="11.6640625" customWidth="1" style="1" min="10" max="11"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="12" max="17"/>
+    <col width="11.6640625" bestFit="1" customWidth="1" style="1" min="18" max="18"/>
+    <col width="9.109375" customWidth="1" style="1" min="19" max="16384"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:10" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="21"/>
-    </row>
-    <row r="4" spans="1:10" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="H4" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4">
+    <row r="2" ht="17.25" customHeight="1" thickBot="1"/>
+    <row r="3" ht="13.8" customHeight="1" thickBot="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Count of Status</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="n"/>
+      <c r="E3" s="20" t="n"/>
+      <c r="F3" s="20" t="n"/>
+      <c r="G3" s="20" t="n"/>
+      <c r="H3" s="20" t="n"/>
+      <c r="I3" s="20" t="n"/>
+      <c r="J3" s="21" t="n"/>
+    </row>
+    <row r="4" ht="13.8" customHeight="1" thickBot="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Scenario Number</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>10 - Not Started</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>20 - In-Process</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>30 - TPR Hold</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>40 - DEV Hold</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>50 - Pass</t>
+        </is>
+      </c>
+      <c r="I4" s="33" t="inlineStr">
+        <is>
+          <t>60 - N/A</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="13.2" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>PP_018</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>RTR</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="6">
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="27">
+    <row r="6" ht="13.2" customHeight="1">
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>PTP</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n"/>
+      <c r="D6" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27">
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="28">
+      <c r="J6" s="28" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="26"/>
-      <c r="B7" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27">
+    <row r="7" ht="13.2" customHeight="1">
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28">
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="28" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
-      <c r="B8" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27">
+    <row r="8" ht="13.8" customHeight="1" thickBot="1">
+      <c r="A8" s="29" t="n"/>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>IMWM</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="J8" s="28">
+      <c r="J8" s="28" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10">
+    <row r="9" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>PP_018 Total</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10">
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="11" t="n">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10">
+    <row r="10" ht="13.8" customHeight="1" thickBot="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>ZZZ999</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="11" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="4">
+    <row r="11" ht="17.25" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>ZZZ999 Total</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="6" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10">
+    <row r="12" ht="13.8" customHeight="1" thickBot="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="11" t="n">
         <v>52</v>
       </c>
     </row>
+    <row r="13" ht="17.25" customHeight="1"/>
+    <row r="14" ht="17.25" customHeight="1"/>
+    <row r="15" ht="17.25" customHeight="1"/>
+    <row r="16" ht="17.25" customHeight="1"/>
+    <row r="17" ht="17.25" customHeight="1"/>
+    <row r="18" ht="17.25" customHeight="1"/>
+    <row r="19" ht="17.25" customHeight="1"/>
+    <row r="20" ht="17.25" customHeight="1"/>
+    <row r="21" ht="17.25" customHeight="1"/>
+    <row r="22" ht="17.25" customHeight="1"/>
+    <row r="23" ht="17.25" customHeight="1"/>
+    <row r="24" ht="17.25" customHeight="1"/>
+    <row r="25" ht="17.25" customHeight="1"/>
+    <row r="26" ht="17.25" customHeight="1"/>
+    <row r="27" ht="17.25" customHeight="1"/>
+    <row r="28" ht="17.25" customHeight="1"/>
+    <row r="29" ht="17.25" customHeight="1"/>
+    <row r="30" ht="17.25" customHeight="1"/>
+    <row r="31" ht="17.25" customHeight="1"/>
+    <row r="32" ht="17.25" customHeight="1"/>
+    <row r="33" ht="17.25" customHeight="1"/>
+    <row r="34" ht="17.25" customHeight="1"/>
+    <row r="35" ht="17.25" customHeight="1"/>
+    <row r="36" ht="17.25" customHeight="1"/>
+    <row r="37" ht="17.25" customHeight="1"/>
+    <row r="38" ht="17.25" customHeight="1"/>
+    <row r="39" ht="17.25" customHeight="1"/>
+    <row r="40" ht="17.25" customHeight="1"/>
+    <row r="41" ht="17.25" customHeight="1"/>
+    <row r="42" ht="17.25" customHeight="1"/>
+    <row r="43" ht="17.25" customHeight="1"/>
+    <row r="44" ht="17.25" customHeight="1"/>
+    <row r="45" ht="17.25" customHeight="1"/>
+    <row r="46" ht="17.25" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>

</xml_diff>